<commit_message>
ajuste no de/para tratamento master plus para opto extra clean
</commit_message>
<xml_diff>
--- a/OPTO_INTEGRATIONS/DB_TRAT.xlsx
+++ b/OPTO_INTEGRATIONS/DB_TRAT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://1masterlabotico-my.sharepoint.com/personal/gustavo_detoni_masterlabotico_com_br/Documents/Área de Trabalho/WMS/OPTO_INTEGRATIONS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_AD4D361C20488DEA4E38A0910C1D7A4A5BDEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3837A328-BC0F-43E9-895A-C0A8670CCEB1}"/>
+  <xr:revisionPtr revIDLastSave="74" documentId="11_AD4D361C20488DEA4E38A0910C1D7A4A5BDEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C70081A-5A2A-4477-ABEF-9B9D970391EB}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -222,11 +222,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,14 +508,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -525,7 +526,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>69286</v>
       </c>
@@ -536,7 +537,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>69285</v>
       </c>
@@ -547,7 +548,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>56405</v>
       </c>
@@ -558,7 +559,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>56716</v>
       </c>
@@ -569,7 +570,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>56407</v>
       </c>
@@ -580,7 +581,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>56406</v>
       </c>
@@ -591,7 +592,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>32</v>
       </c>
@@ -599,10 +600,10 @@
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>70825</v>
       </c>
@@ -613,7 +614,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>56408</v>
       </c>
@@ -624,7 +625,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>69284</v>
       </c>
@@ -635,7 +636,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>57450</v>
       </c>
@@ -646,7 +647,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>68597</v>
       </c>
@@ -657,7 +658,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>57448</v>
       </c>
@@ -667,8 +668,9 @@
       <c r="C14" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="J14" s="2"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>88101</v>
       </c>
@@ -679,7 +681,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>92763</v>
       </c>

</xml_diff>